<commit_message>
corrected user upload format and excel validation added
</commit_message>
<xml_diff>
--- a/public/User_Upload_Template.xlsx
+++ b/public/User_Upload_Template.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="7" documentId="11_085DB817D04A76DEEC5558D754245E3FB48FF27E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2665BDD7-8F0F-4E31-B781-D5675D34FB06}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aditi.s.rajput\Desktop\newProject\newCode\public\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E79B1764-F185-4604-819A-D8A3A06A1792}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1100" yWindow="1100" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -31,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Name</t>
   </si>
@@ -49,13 +54,19 @@
   </si>
   <si>
     <t>Line Manager</t>
+  </si>
+  <si>
+    <t>Franchise</t>
+  </si>
+  <si>
+    <t>Capability</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -411,17 +422,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="25.85546875" customWidth="1"/>
-    <col min="2" max="2" width="20.7109375" customWidth="1"/>
-    <col min="3" max="3" width="25.85546875" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" customWidth="1"/>
-    <col min="5" max="6" width="19.85546875" customWidth="1"/>
+    <col min="1" max="1" width="25.81640625" customWidth="1"/>
+    <col min="2" max="4" width="20.7265625" customWidth="1"/>
+    <col min="5" max="5" width="25.81640625" customWidth="1"/>
+    <col min="6" max="6" width="21.1796875" customWidth="1"/>
+    <col min="7" max="8" width="19.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -429,19 +440,26 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
append to master users file
</commit_message>
<xml_diff>
--- a/public/User_Upload_Template.xlsx
+++ b/public/User_Upload_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aditi.s.rajput\Desktop\newProject\newCode\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E79B1764-F185-4604-819A-D8A3A06A1792}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42C0D62A-FA37-4140-8B05-5EF26CFC2999}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="1100" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -47,19 +47,19 @@
     <t>Level</t>
   </si>
   <si>
-    <t>Location</t>
-  </si>
-  <si>
-    <t>Project</t>
-  </si>
-  <si>
-    <t>Line Manager</t>
-  </si>
-  <si>
     <t>Franchise</t>
   </si>
   <si>
     <t>Capability</t>
+  </si>
+  <si>
+    <t>Work Location</t>
+  </si>
+  <si>
+    <t>Project/Program</t>
+  </si>
+  <si>
+    <t>NWG Line Manager</t>
   </si>
 </sst>
 </file>
@@ -440,22 +440,22 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>